<commit_message>
feat: normaliza nombres de provincias en datos censales
</commit_message>
<xml_diff>
--- a/data/censo_limpio.xlsx
+++ b/data/censo_limpio.xlsx
@@ -443,7 +443,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ciudad Autónoma de Buenos Aires</t>
+          <t>Ciudad Autonoma de Buenos Aires</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -493,7 +493,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Córdoba</t>
+          <t>Cordoba</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -673,7 +673,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tucumán</t>
+          <t>Tucuman</t>
         </is>
       </c>
       <c r="B25" t="n">

</xml_diff>